<commit_message>
Added Find Median From Data Stream Solution
</commit_message>
<xml_diff>
--- a/neetcode_150_tracker.xlsx
+++ b/neetcode_150_tracker.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="203">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -275,6 +275,12 @@
     <t xml:space="preserve">Serialize and Deserialize Binary Tree</t>
   </si>
   <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solved</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tries</t>
   </si>
   <si>
@@ -582,9 +588,6 @@
   </si>
   <si>
     <t xml:space="preserve">Total Problems</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solved</t>
   </si>
   <si>
     <t xml:space="preserve">Attempted (not solved)</t>
@@ -640,7 +643,7 @@
     <numFmt numFmtId="167" formatCode="General"/>
     <numFmt numFmtId="168" formatCode="0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -676,11 +679,6 @@
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="0"/>
     </font>
     <font>
       <b val="true"/>
@@ -792,7 +790,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -853,15 +851,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -873,11 +867,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2776,7 +2770,7 @@
       <c r="I60" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="J60" s="15" t="n">
+      <c r="J60" s="12" t="n">
         <v>46217</v>
       </c>
       <c r="K60" s="10" t="n">
@@ -2799,11 +2793,17 @@
       <c r="D61" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="E61" s="10"/>
-      <c r="F61" s="11"/>
+      <c r="E61" s="10" t="n">
+        <v>46218</v>
+      </c>
+      <c r="F61" s="11" t="s">
+        <v>84</v>
+      </c>
       <c r="G61" s="8"/>
       <c r="H61" s="8"/>
-      <c r="I61" s="11"/>
+      <c r="I61" s="11" t="s">
+        <v>85</v>
+      </c>
       <c r="J61" s="12"/>
       <c r="K61" s="10" t="str">
         <f aca="false">IF(J61="","",J61+14)</f>
@@ -2817,10 +2817,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C62" s="8" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D62" s="13" t="s">
         <v>19</v>
@@ -2843,10 +2843,10 @@
         <v>62</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D63" s="13" t="s">
         <v>19</v>
@@ -2869,10 +2869,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D64" s="14" t="s">
         <v>31</v>
@@ -2895,10 +2895,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D65" s="9" t="s">
         <v>15</v>
@@ -2921,10 +2921,10 @@
         <v>65</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D66" s="9" t="s">
         <v>15</v>
@@ -2947,10 +2947,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D67" s="13" t="s">
         <v>19</v>
@@ -2973,10 +2973,10 @@
         <v>67</v>
       </c>
       <c r="B68" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C68" s="8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D68" s="13" t="s">
         <v>19</v>
@@ -2999,10 +2999,10 @@
         <v>68</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D69" s="13" t="s">
         <v>19</v>
@@ -3025,10 +3025,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C70" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D70" s="13" t="s">
         <v>19</v>
@@ -3051,23 +3051,31 @@
         <v>70</v>
       </c>
       <c r="B71" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D71" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="E71" s="10"/>
-      <c r="F71" s="11"/>
+      <c r="E71" s="10" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F71" s="11" t="s">
+        <v>79</v>
+      </c>
       <c r="G71" s="8"/>
       <c r="H71" s="8"/>
-      <c r="I71" s="11"/>
-      <c r="J71" s="12"/>
-      <c r="K71" s="10" t="str">
+      <c r="I71" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="J71" s="12" t="n">
+        <v>46219</v>
+      </c>
+      <c r="K71" s="10" t="n">
         <f aca="false">IF(J71="","",J71+14)</f>
-        <v/>
+        <v>46233</v>
       </c>
       <c r="L71" s="11"/>
       <c r="M71" s="8"/>
@@ -3077,10 +3085,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D72" s="13" t="s">
         <v>19</v>
@@ -3103,10 +3111,10 @@
         <v>72</v>
       </c>
       <c r="B73" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C73" s="8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D73" s="13" t="s">
         <v>19</v>
@@ -3129,10 +3137,10 @@
         <v>73</v>
       </c>
       <c r="B74" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C74" s="8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D74" s="13" t="s">
         <v>19</v>
@@ -3155,10 +3163,10 @@
         <v>74</v>
       </c>
       <c r="B75" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D75" s="13" t="s">
         <v>19</v>
@@ -3181,10 +3189,10 @@
         <v>75</v>
       </c>
       <c r="B76" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D76" s="13" t="s">
         <v>19</v>
@@ -3207,10 +3215,10 @@
         <v>76</v>
       </c>
       <c r="B77" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D77" s="13" t="s">
         <v>19</v>
@@ -3233,10 +3241,10 @@
         <v>77</v>
       </c>
       <c r="B78" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D78" s="13" t="s">
         <v>19</v>
@@ -3259,10 +3267,10 @@
         <v>78</v>
       </c>
       <c r="B79" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D79" s="13" t="s">
         <v>19</v>
@@ -3285,10 +3293,10 @@
         <v>79</v>
       </c>
       <c r="B80" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C80" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D80" s="14" t="s">
         <v>31</v>
@@ -3311,10 +3319,10 @@
         <v>80</v>
       </c>
       <c r="B81" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C81" s="8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D81" s="13" t="s">
         <v>19</v>
@@ -3337,10 +3345,10 @@
         <v>81</v>
       </c>
       <c r="B82" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C82" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D82" s="13" t="s">
         <v>19</v>
@@ -3363,10 +3371,10 @@
         <v>82</v>
       </c>
       <c r="B83" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C83" s="8" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D83" s="13" t="s">
         <v>19</v>
@@ -3389,10 +3397,10 @@
         <v>83</v>
       </c>
       <c r="B84" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C84" s="8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D84" s="13" t="s">
         <v>19</v>
@@ -3415,10 +3423,10 @@
         <v>84</v>
       </c>
       <c r="B85" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C85" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D85" s="13" t="s">
         <v>19</v>
@@ -3441,10 +3449,10 @@
         <v>85</v>
       </c>
       <c r="B86" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C86" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D86" s="13" t="s">
         <v>19</v>
@@ -3467,10 +3475,10 @@
         <v>86</v>
       </c>
       <c r="B87" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C87" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D87" s="13" t="s">
         <v>19</v>
@@ -3493,10 +3501,10 @@
         <v>87</v>
       </c>
       <c r="B88" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C88" s="8" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D88" s="13" t="s">
         <v>19</v>
@@ -3519,10 +3527,10 @@
         <v>88</v>
       </c>
       <c r="B89" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C89" s="8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D89" s="13" t="s">
         <v>19</v>
@@ -3545,10 +3553,10 @@
         <v>89</v>
       </c>
       <c r="B90" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C90" s="8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D90" s="13" t="s">
         <v>19</v>
@@ -3571,10 +3579,10 @@
         <v>90</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C91" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D91" s="13" t="s">
         <v>19</v>
@@ -3597,10 +3605,10 @@
         <v>91</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C92" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D92" s="13" t="s">
         <v>19</v>
@@ -3623,10 +3631,10 @@
         <v>92</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C93" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D93" s="14" t="s">
         <v>31</v>
@@ -3649,10 +3657,10 @@
         <v>93</v>
       </c>
       <c r="B94" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C94" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D94" s="14" t="s">
         <v>31</v>
@@ -3675,10 +3683,10 @@
         <v>94</v>
       </c>
       <c r="B95" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D95" s="13" t="s">
         <v>19</v>
@@ -3701,10 +3709,10 @@
         <v>95</v>
       </c>
       <c r="B96" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C96" s="8" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D96" s="13" t="s">
         <v>19</v>
@@ -3727,10 +3735,10 @@
         <v>96</v>
       </c>
       <c r="B97" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C97" s="8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D97" s="14" t="s">
         <v>31</v>
@@ -3753,10 +3761,10 @@
         <v>97</v>
       </c>
       <c r="B98" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C98" s="8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D98" s="14" t="s">
         <v>31</v>
@@ -3779,10 +3787,10 @@
         <v>98</v>
       </c>
       <c r="B99" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C99" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D99" s="13" t="s">
         <v>19</v>
@@ -3805,10 +3813,10 @@
         <v>99</v>
       </c>
       <c r="B100" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C100" s="8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D100" s="9" t="s">
         <v>15</v>
@@ -3831,10 +3839,10 @@
         <v>100</v>
       </c>
       <c r="B101" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C101" s="8" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D101" s="9" t="s">
         <v>15</v>
@@ -3857,10 +3865,10 @@
         <v>101</v>
       </c>
       <c r="B102" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C102" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D102" s="13" t="s">
         <v>19</v>
@@ -3883,10 +3891,10 @@
         <v>102</v>
       </c>
       <c r="B103" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C103" s="8" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D103" s="13" t="s">
         <v>19</v>
@@ -3909,10 +3917,10 @@
         <v>103</v>
       </c>
       <c r="B104" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C104" s="8" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D104" s="13" t="s">
         <v>19</v>
@@ -3935,10 +3943,10 @@
         <v>104</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C105" s="8" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D105" s="13" t="s">
         <v>19</v>
@@ -3961,10 +3969,10 @@
         <v>105</v>
       </c>
       <c r="B106" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C106" s="8" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D106" s="13" t="s">
         <v>19</v>
@@ -3987,10 +3995,10 @@
         <v>106</v>
       </c>
       <c r="B107" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C107" s="8" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D107" s="13" t="s">
         <v>19</v>
@@ -4013,10 +4021,10 @@
         <v>107</v>
       </c>
       <c r="B108" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C108" s="8" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D108" s="13" t="s">
         <v>19</v>
@@ -4039,10 +4047,10 @@
         <v>108</v>
       </c>
       <c r="B109" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C109" s="8" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D109" s="13" t="s">
         <v>19</v>
@@ -4065,10 +4073,10 @@
         <v>109</v>
       </c>
       <c r="B110" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C110" s="8" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D110" s="13" t="s">
         <v>19</v>
@@ -4091,10 +4099,10 @@
         <v>110</v>
       </c>
       <c r="B111" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C111" s="8" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D111" s="13" t="s">
         <v>19</v>
@@ -4117,10 +4125,10 @@
         <v>111</v>
       </c>
       <c r="B112" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C112" s="8" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D112" s="13" t="s">
         <v>19</v>
@@ -4143,10 +4151,10 @@
         <v>112</v>
       </c>
       <c r="B113" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C113" s="8" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D113" s="13" t="s">
         <v>19</v>
@@ -4169,10 +4177,10 @@
         <v>113</v>
       </c>
       <c r="B114" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C114" s="8" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D114" s="13" t="s">
         <v>19</v>
@@ -4195,10 +4203,10 @@
         <v>114</v>
       </c>
       <c r="B115" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C115" s="8" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D115" s="13" t="s">
         <v>19</v>
@@ -4221,10 +4229,10 @@
         <v>115</v>
       </c>
       <c r="B116" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C116" s="8" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D116" s="13" t="s">
         <v>19</v>
@@ -4247,10 +4255,10 @@
         <v>116</v>
       </c>
       <c r="B117" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C117" s="8" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D117" s="13" t="s">
         <v>19</v>
@@ -4273,10 +4281,10 @@
         <v>117</v>
       </c>
       <c r="B118" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C118" s="8" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D118" s="14" t="s">
         <v>31</v>
@@ -4299,10 +4307,10 @@
         <v>118</v>
       </c>
       <c r="B119" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C119" s="8" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D119" s="14" t="s">
         <v>31</v>
@@ -4325,10 +4333,10 @@
         <v>119</v>
       </c>
       <c r="B120" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C120" s="8" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D120" s="13" t="s">
         <v>19</v>
@@ -4351,10 +4359,10 @@
         <v>120</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C121" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D121" s="14" t="s">
         <v>31</v>
@@ -4377,10 +4385,10 @@
         <v>121</v>
       </c>
       <c r="B122" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C122" s="8" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D122" s="14" t="s">
         <v>31</v>
@@ -4403,10 +4411,10 @@
         <v>122</v>
       </c>
       <c r="B123" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C123" s="8" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D123" s="13" t="s">
         <v>19</v>
@@ -4429,10 +4437,10 @@
         <v>123</v>
       </c>
       <c r="B124" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D124" s="13" t="s">
         <v>19</v>
@@ -4455,10 +4463,10 @@
         <v>124</v>
       </c>
       <c r="B125" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C125" s="8" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D125" s="13" t="s">
         <v>19</v>
@@ -4481,10 +4489,10 @@
         <v>125</v>
       </c>
       <c r="B126" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D126" s="13" t="s">
         <v>19</v>
@@ -4507,10 +4515,10 @@
         <v>126</v>
       </c>
       <c r="B127" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C127" s="8" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D127" s="13" t="s">
         <v>19</v>
@@ -4533,10 +4541,10 @@
         <v>127</v>
       </c>
       <c r="B128" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C128" s="8" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D128" s="13" t="s">
         <v>19</v>
@@ -4559,10 +4567,10 @@
         <v>128</v>
       </c>
       <c r="B129" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C129" s="8" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D129" s="13" t="s">
         <v>19</v>
@@ -4585,10 +4593,10 @@
         <v>129</v>
       </c>
       <c r="B130" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C130" s="8" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D130" s="13" t="s">
         <v>19</v>
@@ -4611,10 +4619,10 @@
         <v>130</v>
       </c>
       <c r="B131" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C131" s="8" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D131" s="13" t="s">
         <v>19</v>
@@ -4637,10 +4645,10 @@
         <v>131</v>
       </c>
       <c r="B132" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C132" s="8" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D132" s="13" t="s">
         <v>19</v>
@@ -4663,10 +4671,10 @@
         <v>132</v>
       </c>
       <c r="B133" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C133" s="8" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D133" s="13" t="s">
         <v>19</v>
@@ -4689,10 +4697,10 @@
         <v>133</v>
       </c>
       <c r="B134" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C134" s="8" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D134" s="9" t="s">
         <v>15</v>
@@ -4715,10 +4723,10 @@
         <v>134</v>
       </c>
       <c r="B135" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C135" s="8" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D135" s="13" t="s">
         <v>19</v>
@@ -4741,10 +4749,10 @@
         <v>135</v>
       </c>
       <c r="B136" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C136" s="8" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D136" s="14" t="s">
         <v>31</v>
@@ -4767,10 +4775,10 @@
         <v>136</v>
       </c>
       <c r="B137" s="8" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C137" s="8" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D137" s="13" t="s">
         <v>19</v>
@@ -4793,10 +4801,10 @@
         <v>137</v>
       </c>
       <c r="B138" s="8" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C138" s="8" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D138" s="13" t="s">
         <v>19</v>
@@ -4819,10 +4827,10 @@
         <v>138</v>
       </c>
       <c r="B139" s="8" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C139" s="8" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D139" s="13" t="s">
         <v>19</v>
@@ -4845,10 +4853,10 @@
         <v>139</v>
       </c>
       <c r="B140" s="8" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C140" s="8" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D140" s="9" t="s">
         <v>15</v>
@@ -4871,10 +4879,10 @@
         <v>140</v>
       </c>
       <c r="B141" s="8" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C141" s="8" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D141" s="9" t="s">
         <v>15</v>
@@ -4897,10 +4905,10 @@
         <v>141</v>
       </c>
       <c r="B142" s="8" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C142" s="8" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D142" s="13" t="s">
         <v>19</v>
@@ -4923,10 +4931,10 @@
         <v>142</v>
       </c>
       <c r="B143" s="8" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C143" s="8" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D143" s="13" t="s">
         <v>19</v>
@@ -4949,10 +4957,10 @@
         <v>143</v>
       </c>
       <c r="B144" s="8" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C144" s="8" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D144" s="13" t="s">
         <v>19</v>
@@ -4975,10 +4983,10 @@
         <v>144</v>
       </c>
       <c r="B145" s="8" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C145" s="8" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D145" s="9" t="s">
         <v>15</v>
@@ -5001,10 +5009,10 @@
         <v>145</v>
       </c>
       <c r="B146" s="8" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C146" s="8" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D146" s="9" t="s">
         <v>15</v>
@@ -5027,10 +5035,10 @@
         <v>146</v>
       </c>
       <c r="B147" s="8" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C147" s="8" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D147" s="9" t="s">
         <v>15</v>
@@ -5053,10 +5061,10 @@
         <v>147</v>
       </c>
       <c r="B148" s="8" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C148" s="8" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D148" s="9" t="s">
         <v>15</v>
@@ -5079,10 +5087,10 @@
         <v>148</v>
       </c>
       <c r="B149" s="8" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C149" s="8" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D149" s="9" t="s">
         <v>15</v>
@@ -5105,10 +5113,10 @@
         <v>149</v>
       </c>
       <c r="B150" s="8" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C150" s="8" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D150" s="13" t="s">
         <v>19</v>
@@ -5131,10 +5139,10 @@
         <v>150</v>
       </c>
       <c r="B151" s="8" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C151" s="8" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D151" s="13" t="s">
         <v>19</v>
@@ -5209,148 +5217,148 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
-        <v>185</v>
+      <c r="A1" s="15" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="17" t="s">
-        <v>186</v>
-      </c>
-      <c r="B3" s="18" t="n">
+      <c r="A3" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="B3" s="17" t="n">
         <f aca="false">COUNTA(Tracker!C2:C151)</f>
         <v>150</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="s">
-        <v>187</v>
-      </c>
-      <c r="B4" s="18" t="n">
+      <c r="A4" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="17" t="n">
         <f aca="false">COUNTIF(Tracker!I2:I151,"Solved")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="17" t="n">
         <f aca="false">COUNTIF(Tracker!I2:I151,"Solved with Help")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
-        <v>188</v>
-      </c>
-      <c r="B6" s="18" t="n">
+      <c r="A6" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="B6" s="17" t="n">
         <f aca="false">COUNTIF(Tracker!I2:I151,"Attempted")</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
-        <v>189</v>
-      </c>
-      <c r="B7" s="18" t="n">
+      <c r="A7" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="B7" s="17" t="n">
         <f aca="false">COUNTA(Tracker!C2:C151)-COUNTIF(Tracker!I2:I151,"Solved")-COUNTIF(Tracker!I2:I151,"Solved with Help")-COUNTIF(Tracker!I2:I151,"Attempted")</f>
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
-        <v>190</v>
-      </c>
-      <c r="B8" s="19" t="n">
+      <c r="A8" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="B8" s="18" t="n">
         <f aca="false">(COUNTIF(Tracker!I2:I151,"Solved")+COUNTIF(Tracker!I2:I151,"Solved with Help"))/COUNTA(Tracker!C2:C151)</f>
-        <v>0.02</v>
+        <v>0.0333333333333333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
-        <v>191</v>
-      </c>
-      <c r="B9" s="18" t="n">
+      <c r="A9" s="16" t="s">
+        <v>192</v>
+      </c>
+      <c r="B9" s="17" t="n">
         <f aca="true">COUNTIFS(Tracker!K2:K151,"&lt;="&amp;TODAY(),Tracker!K2:K151,"&lt;&gt;",Tracker!L2:L151,"&lt;&gt;Yes")</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
-        <v>192</v>
+      <c r="A11" s="19" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="18" t="str">
+      <c r="B12" s="17" t="str">
         <f aca="false">COUNTIFS(Tracker!D2:D151,"Easy",Tracker!I2:I151,"Solved")&amp;"/"&amp;COUNTIF(Tracker!D2:D151,"Easy")</f>
         <v>0/28</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="18" t="str">
+      <c r="A13" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="17" t="str">
         <f aca="false">COUNTIFS(Tracker!D2:D151,"Medium",Tracker!I2:I151,"Solved")&amp;"/"&amp;COUNTIF(Tracker!D2:D151,"Medium")</f>
         <v>0/101</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="18" t="str">
+      <c r="B14" s="17" t="str">
         <f aca="false">COUNTIFS(Tracker!D2:D151,"Hard",Tracker!I2:I151,"Solved")&amp;"/"&amp;COUNTIF(Tracker!D2:D151,"Hard")</f>
-        <v>0/21</v>
+        <v>1/21</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
-        <v>193</v>
+      <c r="A16" s="19" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="s">
-        <v>194</v>
+      <c r="A17" s="20" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="s">
-        <v>195</v>
+      <c r="A18" s="20" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="s">
-        <v>196</v>
+      <c r="A19" s="20" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
-        <v>197</v>
+      <c r="A20" s="20" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
-        <v>198</v>
+      <c r="A21" s="20" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
-        <v>199</v>
+      <c r="A22" s="20" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
-        <v>200</v>
+      <c r="A23" s="20" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
-        <v>201</v>
+      <c r="A24" s="20" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Word Search Solution
</commit_message>
<xml_diff>
--- a/neetcode_150_tracker.xlsx
+++ b/neetcode_150_tracker.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="204">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -263,24 +263,24 @@
     <t xml:space="preserve">No</t>
   </si>
   <si>
+    <t xml:space="preserve">Solved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Construct Binary Tree from Preorder and Inorder Traversal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binary Tree Maximum Path Sum</t>
+  </si>
+  <si>
     <t xml:space="preserve">Solved with Help</t>
   </si>
   <si>
-    <t xml:space="preserve">Construct Binary Tree from Preorder and Inorder Traversal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Binary Tree Maximum Path Sum</t>
-  </si>
-  <si>
     <t xml:space="preserve">Serialize and Deserialize Binary Tree</t>
   </si>
   <si>
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
-    <t xml:space="preserve">Solved</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tries</t>
   </si>
   <si>
@@ -336,6 +336,9 @@
   </si>
   <si>
     <t xml:space="preserve">Word Search</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28,Jul,2026</t>
   </si>
   <si>
     <t xml:space="preserve">Palindrome Partitioning</t>
@@ -2702,12 +2705,10 @@
       <c r="I58" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="J58" s="12" t="n">
-        <v>46213</v>
-      </c>
-      <c r="K58" s="10" t="n">
+      <c r="J58" s="12"/>
+      <c r="K58" s="10" t="str">
         <f aca="false">IF(J58="","",J58+14)</f>
-        <v>46227</v>
+        <v/>
       </c>
       <c r="L58" s="11"/>
       <c r="M58" s="8"/>
@@ -2736,12 +2737,10 @@
       <c r="I59" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="J59" s="12" t="n">
-        <v>46214</v>
-      </c>
-      <c r="K59" s="10" t="n">
+      <c r="J59" s="12"/>
+      <c r="K59" s="10" t="str">
         <f aca="false">IF(J59="","",J59+14)</f>
-        <v>46228</v>
+        <v/>
       </c>
       <c r="L59" s="11"/>
       <c r="M59" s="8"/>
@@ -2768,7 +2767,7 @@
       <c r="G60" s="8"/>
       <c r="H60" s="8"/>
       <c r="I60" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="J60" s="12" t="n">
         <v>46217</v>
@@ -2788,7 +2787,7 @@
         <v>66</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D61" s="14" t="s">
         <v>31</v>
@@ -2797,12 +2796,12 @@
         <v>46218</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G61" s="8"/>
       <c r="H61" s="8"/>
       <c r="I61" s="11" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="J61" s="12"/>
       <c r="K61" s="10" t="str">
@@ -3070,12 +3069,10 @@
       <c r="I71" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="J71" s="12" t="n">
-        <v>46219</v>
-      </c>
-      <c r="K71" s="10" t="n">
+      <c r="J71" s="12"/>
+      <c r="K71" s="10" t="str">
         <f aca="false">IF(J71="","",J71+14)</f>
-        <v>46233</v>
+        <v/>
       </c>
       <c r="L71" s="11"/>
       <c r="M71" s="8"/>
@@ -3119,15 +3116,23 @@
       <c r="D73" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E73" s="10"/>
-      <c r="F73" s="11"/>
+      <c r="E73" s="10" t="n">
+        <v>46221</v>
+      </c>
+      <c r="F73" s="11" t="s">
+        <v>79</v>
+      </c>
       <c r="G73" s="8"/>
       <c r="H73" s="8"/>
-      <c r="I73" s="11"/>
-      <c r="J73" s="12"/>
-      <c r="K73" s="10" t="str">
+      <c r="I73" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="J73" s="12" t="n">
+        <v>46221</v>
+      </c>
+      <c r="K73" s="10" t="n">
         <f aca="false">IF(J73="","",J73+14)</f>
-        <v/>
+        <v>46235</v>
       </c>
       <c r="L73" s="11"/>
       <c r="M73" s="8"/>
@@ -3223,15 +3228,23 @@
       <c r="D77" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E77" s="10"/>
-      <c r="F77" s="11"/>
+      <c r="E77" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="F77" s="11" t="s">
+        <v>79</v>
+      </c>
       <c r="G77" s="8"/>
       <c r="H77" s="8"/>
-      <c r="I77" s="11"/>
-      <c r="J77" s="12"/>
-      <c r="K77" s="10" t="str">
+      <c r="I77" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="J77" s="12" t="n">
+        <v>46231</v>
+      </c>
+      <c r="K77" s="10" t="n">
         <f aca="false">IF(J77="","",J77+14)</f>
-        <v/>
+        <v>46245</v>
       </c>
       <c r="L77" s="11"/>
       <c r="M77" s="8"/>
@@ -3244,7 +3257,7 @@
         <v>98</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D78" s="13" t="s">
         <v>19</v>
@@ -3270,7 +3283,7 @@
         <v>98</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D79" s="13" t="s">
         <v>19</v>
@@ -3296,7 +3309,7 @@
         <v>98</v>
       </c>
       <c r="C80" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D80" s="14" t="s">
         <v>31</v>
@@ -3319,10 +3332,10 @@
         <v>80</v>
       </c>
       <c r="B81" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C81" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D81" s="13" t="s">
         <v>19</v>
@@ -3345,10 +3358,10 @@
         <v>81</v>
       </c>
       <c r="B82" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C82" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D82" s="13" t="s">
         <v>19</v>
@@ -3371,10 +3384,10 @@
         <v>82</v>
       </c>
       <c r="B83" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C83" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D83" s="13" t="s">
         <v>19</v>
@@ -3397,10 +3410,10 @@
         <v>83</v>
       </c>
       <c r="B84" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C84" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D84" s="13" t="s">
         <v>19</v>
@@ -3423,10 +3436,10 @@
         <v>84</v>
       </c>
       <c r="B85" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C85" s="8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D85" s="13" t="s">
         <v>19</v>
@@ -3449,10 +3462,10 @@
         <v>85</v>
       </c>
       <c r="B86" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C86" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D86" s="13" t="s">
         <v>19</v>
@@ -3475,10 +3488,10 @@
         <v>86</v>
       </c>
       <c r="B87" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C87" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D87" s="13" t="s">
         <v>19</v>
@@ -3501,10 +3514,10 @@
         <v>87</v>
       </c>
       <c r="B88" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C88" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D88" s="13" t="s">
         <v>19</v>
@@ -3527,10 +3540,10 @@
         <v>88</v>
       </c>
       <c r="B89" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C89" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D89" s="13" t="s">
         <v>19</v>
@@ -3553,10 +3566,10 @@
         <v>89</v>
       </c>
       <c r="B90" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C90" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D90" s="13" t="s">
         <v>19</v>
@@ -3579,10 +3592,10 @@
         <v>90</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C91" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D91" s="13" t="s">
         <v>19</v>
@@ -3605,10 +3618,10 @@
         <v>91</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C92" s="8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D92" s="13" t="s">
         <v>19</v>
@@ -3631,10 +3644,10 @@
         <v>92</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C93" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D93" s="14" t="s">
         <v>31</v>
@@ -3657,10 +3670,10 @@
         <v>93</v>
       </c>
       <c r="B94" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C94" s="8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D94" s="14" t="s">
         <v>31</v>
@@ -3683,10 +3696,10 @@
         <v>94</v>
       </c>
       <c r="B95" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D95" s="13" t="s">
         <v>19</v>
@@ -3709,10 +3722,10 @@
         <v>95</v>
       </c>
       <c r="B96" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C96" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D96" s="13" t="s">
         <v>19</v>
@@ -3735,10 +3748,10 @@
         <v>96</v>
       </c>
       <c r="B97" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C97" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D97" s="14" t="s">
         <v>31</v>
@@ -3761,10 +3774,10 @@
         <v>97</v>
       </c>
       <c r="B98" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C98" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D98" s="14" t="s">
         <v>31</v>
@@ -3787,10 +3800,10 @@
         <v>98</v>
       </c>
       <c r="B99" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C99" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D99" s="13" t="s">
         <v>19</v>
@@ -3813,10 +3826,10 @@
         <v>99</v>
       </c>
       <c r="B100" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C100" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D100" s="9" t="s">
         <v>15</v>
@@ -3839,10 +3852,10 @@
         <v>100</v>
       </c>
       <c r="B101" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C101" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D101" s="9" t="s">
         <v>15</v>
@@ -3865,10 +3878,10 @@
         <v>101</v>
       </c>
       <c r="B102" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C102" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D102" s="13" t="s">
         <v>19</v>
@@ -3891,10 +3904,10 @@
         <v>102</v>
       </c>
       <c r="B103" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C103" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D103" s="13" t="s">
         <v>19</v>
@@ -3917,10 +3930,10 @@
         <v>103</v>
       </c>
       <c r="B104" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C104" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D104" s="13" t="s">
         <v>19</v>
@@ -3943,10 +3956,10 @@
         <v>104</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C105" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D105" s="13" t="s">
         <v>19</v>
@@ -3969,10 +3982,10 @@
         <v>105</v>
       </c>
       <c r="B106" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C106" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D106" s="13" t="s">
         <v>19</v>
@@ -3995,10 +4008,10 @@
         <v>106</v>
       </c>
       <c r="B107" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C107" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D107" s="13" t="s">
         <v>19</v>
@@ -4021,10 +4034,10 @@
         <v>107</v>
       </c>
       <c r="B108" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C108" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D108" s="13" t="s">
         <v>19</v>
@@ -4047,10 +4060,10 @@
         <v>108</v>
       </c>
       <c r="B109" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C109" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D109" s="13" t="s">
         <v>19</v>
@@ -4073,10 +4086,10 @@
         <v>109</v>
       </c>
       <c r="B110" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C110" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D110" s="13" t="s">
         <v>19</v>
@@ -4099,10 +4112,10 @@
         <v>110</v>
       </c>
       <c r="B111" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C111" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D111" s="13" t="s">
         <v>19</v>
@@ -4125,10 +4138,10 @@
         <v>111</v>
       </c>
       <c r="B112" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C112" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D112" s="13" t="s">
         <v>19</v>
@@ -4151,10 +4164,10 @@
         <v>112</v>
       </c>
       <c r="B113" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C113" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D113" s="13" t="s">
         <v>19</v>
@@ -4177,10 +4190,10 @@
         <v>113</v>
       </c>
       <c r="B114" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C114" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D114" s="13" t="s">
         <v>19</v>
@@ -4203,10 +4216,10 @@
         <v>114</v>
       </c>
       <c r="B115" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C115" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D115" s="13" t="s">
         <v>19</v>
@@ -4229,10 +4242,10 @@
         <v>115</v>
       </c>
       <c r="B116" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C116" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D116" s="13" t="s">
         <v>19</v>
@@ -4255,10 +4268,10 @@
         <v>116</v>
       </c>
       <c r="B117" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C117" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D117" s="13" t="s">
         <v>19</v>
@@ -4281,10 +4294,10 @@
         <v>117</v>
       </c>
       <c r="B118" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C118" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D118" s="14" t="s">
         <v>31</v>
@@ -4307,10 +4320,10 @@
         <v>118</v>
       </c>
       <c r="B119" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C119" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D119" s="14" t="s">
         <v>31</v>
@@ -4333,10 +4346,10 @@
         <v>119</v>
       </c>
       <c r="B120" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C120" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D120" s="13" t="s">
         <v>19</v>
@@ -4359,10 +4372,10 @@
         <v>120</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C121" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D121" s="14" t="s">
         <v>31</v>
@@ -4385,10 +4398,10 @@
         <v>121</v>
       </c>
       <c r="B122" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C122" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D122" s="14" t="s">
         <v>31</v>
@@ -4411,10 +4424,10 @@
         <v>122</v>
       </c>
       <c r="B123" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C123" s="8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D123" s="13" t="s">
         <v>19</v>
@@ -4437,10 +4450,10 @@
         <v>123</v>
       </c>
       <c r="B124" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D124" s="13" t="s">
         <v>19</v>
@@ -4463,10 +4476,10 @@
         <v>124</v>
       </c>
       <c r="B125" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C125" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D125" s="13" t="s">
         <v>19</v>
@@ -4489,10 +4502,10 @@
         <v>125</v>
       </c>
       <c r="B126" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D126" s="13" t="s">
         <v>19</v>
@@ -4515,10 +4528,10 @@
         <v>126</v>
       </c>
       <c r="B127" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C127" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D127" s="13" t="s">
         <v>19</v>
@@ -4541,10 +4554,10 @@
         <v>127</v>
       </c>
       <c r="B128" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C128" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D128" s="13" t="s">
         <v>19</v>
@@ -4567,10 +4580,10 @@
         <v>128</v>
       </c>
       <c r="B129" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C129" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D129" s="13" t="s">
         <v>19</v>
@@ -4593,10 +4606,10 @@
         <v>129</v>
       </c>
       <c r="B130" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C130" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D130" s="13" t="s">
         <v>19</v>
@@ -4619,10 +4632,10 @@
         <v>130</v>
       </c>
       <c r="B131" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C131" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D131" s="13" t="s">
         <v>19</v>
@@ -4645,10 +4658,10 @@
         <v>131</v>
       </c>
       <c r="B132" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C132" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D132" s="13" t="s">
         <v>19</v>
@@ -4671,10 +4684,10 @@
         <v>132</v>
       </c>
       <c r="B133" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C133" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D133" s="13" t="s">
         <v>19</v>
@@ -4697,10 +4710,10 @@
         <v>133</v>
       </c>
       <c r="B134" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C134" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D134" s="9" t="s">
         <v>15</v>
@@ -4723,10 +4736,10 @@
         <v>134</v>
       </c>
       <c r="B135" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C135" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D135" s="13" t="s">
         <v>19</v>
@@ -4749,10 +4762,10 @@
         <v>135</v>
       </c>
       <c r="B136" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C136" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D136" s="14" t="s">
         <v>31</v>
@@ -4775,10 +4788,10 @@
         <v>136</v>
       </c>
       <c r="B137" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C137" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D137" s="13" t="s">
         <v>19</v>
@@ -4801,10 +4814,10 @@
         <v>137</v>
       </c>
       <c r="B138" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C138" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D138" s="13" t="s">
         <v>19</v>
@@ -4827,10 +4840,10 @@
         <v>138</v>
       </c>
       <c r="B139" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C139" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D139" s="13" t="s">
         <v>19</v>
@@ -4853,10 +4866,10 @@
         <v>139</v>
       </c>
       <c r="B140" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C140" s="8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D140" s="9" t="s">
         <v>15</v>
@@ -4879,10 +4892,10 @@
         <v>140</v>
       </c>
       <c r="B141" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C141" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D141" s="9" t="s">
         <v>15</v>
@@ -4905,10 +4918,10 @@
         <v>141</v>
       </c>
       <c r="B142" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C142" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D142" s="13" t="s">
         <v>19</v>
@@ -4931,10 +4944,10 @@
         <v>142</v>
       </c>
       <c r="B143" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C143" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D143" s="13" t="s">
         <v>19</v>
@@ -4957,10 +4970,10 @@
         <v>143</v>
       </c>
       <c r="B144" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C144" s="8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D144" s="13" t="s">
         <v>19</v>
@@ -4983,10 +4996,10 @@
         <v>144</v>
       </c>
       <c r="B145" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C145" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D145" s="9" t="s">
         <v>15</v>
@@ -5009,10 +5022,10 @@
         <v>145</v>
       </c>
       <c r="B146" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C146" s="8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D146" s="9" t="s">
         <v>15</v>
@@ -5035,10 +5048,10 @@
         <v>146</v>
       </c>
       <c r="B147" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C147" s="8" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D147" s="9" t="s">
         <v>15</v>
@@ -5061,10 +5074,10 @@
         <v>147</v>
       </c>
       <c r="B148" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C148" s="8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D148" s="9" t="s">
         <v>15</v>
@@ -5087,10 +5100,10 @@
         <v>148</v>
       </c>
       <c r="B149" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C149" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D149" s="9" t="s">
         <v>15</v>
@@ -5113,10 +5126,10 @@
         <v>149</v>
       </c>
       <c r="B150" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C150" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D150" s="13" t="s">
         <v>19</v>
@@ -5139,10 +5152,10 @@
         <v>150</v>
       </c>
       <c r="B151" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C151" s="8" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D151" s="13" t="s">
         <v>19</v>
@@ -5218,12 +5231,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B3" s="17" t="n">
         <f aca="false">COUNTA(Tracker!C2:C151)</f>
@@ -5232,25 +5245,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B4" s="17" t="n">
         <f aca="false">COUNTIF(Tracker!I2:I151,"Solved")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B5" s="17" t="n">
         <f aca="false">COUNTIF(Tracker!I2:I151,"Solved with Help")</f>
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B6" s="17" t="n">
         <f aca="false">COUNTIF(Tracker!I2:I151,"Attempted")</f>
@@ -5259,34 +5272,34 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B7" s="17" t="n">
         <f aca="false">COUNTA(Tracker!C2:C151)-COUNTIF(Tracker!I2:I151,"Solved")-COUNTIF(Tracker!I2:I151,"Solved with Help")-COUNTIF(Tracker!I2:I151,"Attempted")</f>
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B8" s="18" t="n">
         <f aca="false">(COUNTIF(Tracker!I2:I151,"Solved")+COUNTIF(Tracker!I2:I151,"Solved with Help"))/COUNTA(Tracker!C2:C151)</f>
-        <v>0.0333333333333333</v>
+        <v>0.0466666666666667</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B9" s="17" t="n">
         <f aca="true">COUNTIFS(Tracker!K2:K151,"&lt;="&amp;TODAY(),Tracker!K2:K151,"&lt;&gt;",Tracker!L2:L151,"&lt;&gt;Yes")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5304,7 +5317,7 @@
       </c>
       <c r="B13" s="17" t="str">
         <f aca="false">COUNTIFS(Tracker!D2:D151,"Medium",Tracker!I2:I151,"Solved")&amp;"/"&amp;COUNTIF(Tracker!D2:D151,"Medium")</f>
-        <v>0/101</v>
+        <v>3/101</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5313,52 +5326,52 @@
       </c>
       <c r="B14" s="17" t="str">
         <f aca="false">COUNTIFS(Tracker!D2:D151,"Hard",Tracker!I2:I151,"Solved")&amp;"/"&amp;COUNTIF(Tracker!D2:D151,"Hard")</f>
-        <v>1/21</v>
+        <v>2/21</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Implement Trie Solution
</commit_message>
<xml_diff>
--- a/neetcode_150_tracker.xlsx
+++ b/neetcode_150_tracker.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Tracker" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="203">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -336,9 +336,6 @@
   </si>
   <si>
     <t xml:space="preserve">Word Search</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28,Jul,2026</t>
   </si>
   <si>
     <t xml:space="preserve">Palindrome Partitioning</t>
@@ -2824,15 +2821,22 @@
       <c r="D62" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E62" s="10"/>
-      <c r="F62" s="11"/>
+      <c r="E62" s="10" t="n">
+        <v>46233</v>
+      </c>
+      <c r="F62" s="11" t="s">
+        <v>79</v>
+      </c>
       <c r="G62" s="8"/>
       <c r="H62" s="8"/>
-      <c r="I62" s="11"/>
-      <c r="J62" s="12"/>
-      <c r="K62" s="10" t="str">
-        <f aca="false">IF(J62="","",J62+14)</f>
-        <v/>
+      <c r="I62" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="J62" s="12" t="n">
+        <v>46221</v>
+      </c>
+      <c r="K62" s="10" t="n">
+        <v>46247</v>
       </c>
       <c r="L62" s="11"/>
       <c r="M62" s="8"/>
@@ -2856,10 +2860,7 @@
       <c r="H63" s="8"/>
       <c r="I63" s="11"/>
       <c r="J63" s="12"/>
-      <c r="K63" s="10" t="str">
-        <f aca="false">IF(J63="","",J63+14)</f>
-        <v/>
-      </c>
+      <c r="K63" s="10"/>
       <c r="L63" s="11"/>
       <c r="M63" s="8"/>
     </row>
@@ -2882,10 +2883,7 @@
       <c r="H64" s="8"/>
       <c r="I64" s="11"/>
       <c r="J64" s="12"/>
-      <c r="K64" s="10" t="str">
-        <f aca="false">IF(J64="","",J64+14)</f>
-        <v/>
-      </c>
+      <c r="K64" s="10"/>
       <c r="L64" s="11"/>
       <c r="M64" s="8"/>
     </row>
@@ -3228,8 +3226,8 @@
       <c r="D77" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E77" s="10" t="s">
-        <v>105</v>
+      <c r="E77" s="10" t="n">
+        <v>46231</v>
       </c>
       <c r="F77" s="11" t="s">
         <v>79</v>
@@ -3257,7 +3255,7 @@
         <v>98</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D78" s="13" t="s">
         <v>19</v>
@@ -3283,7 +3281,7 @@
         <v>98</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D79" s="13" t="s">
         <v>19</v>
@@ -3309,7 +3307,7 @@
         <v>98</v>
       </c>
       <c r="C80" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D80" s="14" t="s">
         <v>31</v>
@@ -3332,10 +3330,10 @@
         <v>80</v>
       </c>
       <c r="B81" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C81" s="8" t="s">
         <v>109</v>
-      </c>
-      <c r="C81" s="8" t="s">
-        <v>110</v>
       </c>
       <c r="D81" s="13" t="s">
         <v>19</v>
@@ -3358,10 +3356,10 @@
         <v>81</v>
       </c>
       <c r="B82" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C82" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D82" s="13" t="s">
         <v>19</v>
@@ -3384,10 +3382,10 @@
         <v>82</v>
       </c>
       <c r="B83" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C83" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D83" s="13" t="s">
         <v>19</v>
@@ -3410,10 +3408,10 @@
         <v>83</v>
       </c>
       <c r="B84" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C84" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D84" s="13" t="s">
         <v>19</v>
@@ -3436,10 +3434,10 @@
         <v>84</v>
       </c>
       <c r="B85" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C85" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D85" s="13" t="s">
         <v>19</v>
@@ -3462,10 +3460,10 @@
         <v>85</v>
       </c>
       <c r="B86" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C86" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D86" s="13" t="s">
         <v>19</v>
@@ -3488,10 +3486,10 @@
         <v>86</v>
       </c>
       <c r="B87" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C87" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D87" s="13" t="s">
         <v>19</v>
@@ -3514,10 +3512,10 @@
         <v>87</v>
       </c>
       <c r="B88" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C88" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D88" s="13" t="s">
         <v>19</v>
@@ -3540,10 +3538,10 @@
         <v>88</v>
       </c>
       <c r="B89" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C89" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D89" s="13" t="s">
         <v>19</v>
@@ -3566,10 +3564,10 @@
         <v>89</v>
       </c>
       <c r="B90" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C90" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D90" s="13" t="s">
         <v>19</v>
@@ -3592,10 +3590,10 @@
         <v>90</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C91" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D91" s="13" t="s">
         <v>19</v>
@@ -3618,10 +3616,10 @@
         <v>91</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C92" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D92" s="13" t="s">
         <v>19</v>
@@ -3644,10 +3642,10 @@
         <v>92</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C93" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D93" s="14" t="s">
         <v>31</v>
@@ -3670,10 +3668,10 @@
         <v>93</v>
       </c>
       <c r="B94" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C94" s="8" t="s">
         <v>123</v>
-      </c>
-      <c r="C94" s="8" t="s">
-        <v>124</v>
       </c>
       <c r="D94" s="14" t="s">
         <v>31</v>
@@ -3696,10 +3694,10 @@
         <v>94</v>
       </c>
       <c r="B95" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D95" s="13" t="s">
         <v>19</v>
@@ -3722,10 +3720,10 @@
         <v>95</v>
       </c>
       <c r="B96" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C96" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D96" s="13" t="s">
         <v>19</v>
@@ -3748,10 +3746,10 @@
         <v>96</v>
       </c>
       <c r="B97" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C97" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D97" s="14" t="s">
         <v>31</v>
@@ -3774,10 +3772,10 @@
         <v>97</v>
       </c>
       <c r="B98" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C98" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D98" s="14" t="s">
         <v>31</v>
@@ -3800,10 +3798,10 @@
         <v>98</v>
       </c>
       <c r="B99" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C99" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D99" s="13" t="s">
         <v>19</v>
@@ -3826,10 +3824,10 @@
         <v>99</v>
       </c>
       <c r="B100" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C100" s="8" t="s">
         <v>130</v>
-      </c>
-      <c r="C100" s="8" t="s">
-        <v>131</v>
       </c>
       <c r="D100" s="9" t="s">
         <v>15</v>
@@ -3852,10 +3850,10 @@
         <v>100</v>
       </c>
       <c r="B101" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C101" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D101" s="9" t="s">
         <v>15</v>
@@ -3878,10 +3876,10 @@
         <v>101</v>
       </c>
       <c r="B102" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C102" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D102" s="13" t="s">
         <v>19</v>
@@ -3904,10 +3902,10 @@
         <v>102</v>
       </c>
       <c r="B103" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C103" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D103" s="13" t="s">
         <v>19</v>
@@ -3930,10 +3928,10 @@
         <v>103</v>
       </c>
       <c r="B104" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C104" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D104" s="13" t="s">
         <v>19</v>
@@ -3956,10 +3954,10 @@
         <v>104</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C105" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D105" s="13" t="s">
         <v>19</v>
@@ -3982,10 +3980,10 @@
         <v>105</v>
       </c>
       <c r="B106" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C106" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D106" s="13" t="s">
         <v>19</v>
@@ -4008,10 +4006,10 @@
         <v>106</v>
       </c>
       <c r="B107" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C107" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D107" s="13" t="s">
         <v>19</v>
@@ -4034,10 +4032,10 @@
         <v>107</v>
       </c>
       <c r="B108" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C108" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D108" s="13" t="s">
         <v>19</v>
@@ -4060,10 +4058,10 @@
         <v>108</v>
       </c>
       <c r="B109" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C109" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D109" s="13" t="s">
         <v>19</v>
@@ -4086,10 +4084,10 @@
         <v>109</v>
       </c>
       <c r="B110" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C110" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D110" s="13" t="s">
         <v>19</v>
@@ -4112,10 +4110,10 @@
         <v>110</v>
       </c>
       <c r="B111" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C111" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D111" s="13" t="s">
         <v>19</v>
@@ -4138,10 +4136,10 @@
         <v>111</v>
       </c>
       <c r="B112" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C112" s="8" t="s">
         <v>143</v>
-      </c>
-      <c r="C112" s="8" t="s">
-        <v>144</v>
       </c>
       <c r="D112" s="13" t="s">
         <v>19</v>
@@ -4164,10 +4162,10 @@
         <v>112</v>
       </c>
       <c r="B113" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C113" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D113" s="13" t="s">
         <v>19</v>
@@ -4190,10 +4188,10 @@
         <v>113</v>
       </c>
       <c r="B114" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C114" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D114" s="13" t="s">
         <v>19</v>
@@ -4216,10 +4214,10 @@
         <v>114</v>
       </c>
       <c r="B115" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C115" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D115" s="13" t="s">
         <v>19</v>
@@ -4242,10 +4240,10 @@
         <v>115</v>
       </c>
       <c r="B116" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C116" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D116" s="13" t="s">
         <v>19</v>
@@ -4268,10 +4266,10 @@
         <v>116</v>
       </c>
       <c r="B117" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C117" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D117" s="13" t="s">
         <v>19</v>
@@ -4294,10 +4292,10 @@
         <v>117</v>
       </c>
       <c r="B118" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C118" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D118" s="14" t="s">
         <v>31</v>
@@ -4320,10 +4318,10 @@
         <v>118</v>
       </c>
       <c r="B119" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C119" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D119" s="14" t="s">
         <v>31</v>
@@ -4346,10 +4344,10 @@
         <v>119</v>
       </c>
       <c r="B120" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C120" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D120" s="13" t="s">
         <v>19</v>
@@ -4372,10 +4370,10 @@
         <v>120</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C121" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D121" s="14" t="s">
         <v>31</v>
@@ -4398,10 +4396,10 @@
         <v>121</v>
       </c>
       <c r="B122" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C122" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D122" s="14" t="s">
         <v>31</v>
@@ -4424,10 +4422,10 @@
         <v>122</v>
       </c>
       <c r="B123" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C123" s="8" t="s">
         <v>155</v>
-      </c>
-      <c r="C123" s="8" t="s">
-        <v>156</v>
       </c>
       <c r="D123" s="13" t="s">
         <v>19</v>
@@ -4450,10 +4448,10 @@
         <v>123</v>
       </c>
       <c r="B124" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D124" s="13" t="s">
         <v>19</v>
@@ -4476,10 +4474,10 @@
         <v>124</v>
       </c>
       <c r="B125" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C125" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D125" s="13" t="s">
         <v>19</v>
@@ -4502,10 +4500,10 @@
         <v>125</v>
       </c>
       <c r="B126" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D126" s="13" t="s">
         <v>19</v>
@@ -4528,10 +4526,10 @@
         <v>126</v>
       </c>
       <c r="B127" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C127" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D127" s="13" t="s">
         <v>19</v>
@@ -4554,10 +4552,10 @@
         <v>127</v>
       </c>
       <c r="B128" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C128" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D128" s="13" t="s">
         <v>19</v>
@@ -4580,10 +4578,10 @@
         <v>128</v>
       </c>
       <c r="B129" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C129" s="8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D129" s="13" t="s">
         <v>19</v>
@@ -4606,10 +4604,10 @@
         <v>129</v>
       </c>
       <c r="B130" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C130" s="8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D130" s="13" t="s">
         <v>19</v>
@@ -4632,10 +4630,10 @@
         <v>130</v>
       </c>
       <c r="B131" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="C131" s="8" t="s">
         <v>164</v>
-      </c>
-      <c r="C131" s="8" t="s">
-        <v>165</v>
       </c>
       <c r="D131" s="13" t="s">
         <v>19</v>
@@ -4658,10 +4656,10 @@
         <v>131</v>
       </c>
       <c r="B132" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C132" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D132" s="13" t="s">
         <v>19</v>
@@ -4684,10 +4682,10 @@
         <v>132</v>
       </c>
       <c r="B133" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C133" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D133" s="13" t="s">
         <v>19</v>
@@ -4710,10 +4708,10 @@
         <v>133</v>
       </c>
       <c r="B134" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C134" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D134" s="9" t="s">
         <v>15</v>
@@ -4736,10 +4734,10 @@
         <v>134</v>
       </c>
       <c r="B135" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C135" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D135" s="13" t="s">
         <v>19</v>
@@ -4762,10 +4760,10 @@
         <v>135</v>
       </c>
       <c r="B136" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C136" s="8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D136" s="14" t="s">
         <v>31</v>
@@ -4788,10 +4786,10 @@
         <v>136</v>
       </c>
       <c r="B137" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C137" s="8" t="s">
         <v>171</v>
-      </c>
-      <c r="C137" s="8" t="s">
-        <v>172</v>
       </c>
       <c r="D137" s="13" t="s">
         <v>19</v>
@@ -4814,10 +4812,10 @@
         <v>137</v>
       </c>
       <c r="B138" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C138" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D138" s="13" t="s">
         <v>19</v>
@@ -4840,10 +4838,10 @@
         <v>138</v>
       </c>
       <c r="B139" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C139" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D139" s="13" t="s">
         <v>19</v>
@@ -4866,10 +4864,10 @@
         <v>139</v>
       </c>
       <c r="B140" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C140" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D140" s="9" t="s">
         <v>15</v>
@@ -4892,10 +4890,10 @@
         <v>140</v>
       </c>
       <c r="B141" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C141" s="8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D141" s="9" t="s">
         <v>15</v>
@@ -4918,10 +4916,10 @@
         <v>141</v>
       </c>
       <c r="B142" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C142" s="8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D142" s="13" t="s">
         <v>19</v>
@@ -4944,10 +4942,10 @@
         <v>142</v>
       </c>
       <c r="B143" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C143" s="8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D143" s="13" t="s">
         <v>19</v>
@@ -4970,10 +4968,10 @@
         <v>143</v>
       </c>
       <c r="B144" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C144" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D144" s="13" t="s">
         <v>19</v>
@@ -4996,10 +4994,10 @@
         <v>144</v>
       </c>
       <c r="B145" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="C145" s="8" t="s">
         <v>180</v>
-      </c>
-      <c r="C145" s="8" t="s">
-        <v>181</v>
       </c>
       <c r="D145" s="9" t="s">
         <v>15</v>
@@ -5022,10 +5020,10 @@
         <v>145</v>
       </c>
       <c r="B146" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C146" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D146" s="9" t="s">
         <v>15</v>
@@ -5048,10 +5046,10 @@
         <v>146</v>
       </c>
       <c r="B147" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C147" s="8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D147" s="9" t="s">
         <v>15</v>
@@ -5074,10 +5072,10 @@
         <v>147</v>
       </c>
       <c r="B148" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C148" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D148" s="9" t="s">
         <v>15</v>
@@ -5100,10 +5098,10 @@
         <v>148</v>
       </c>
       <c r="B149" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C149" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D149" s="9" t="s">
         <v>15</v>
@@ -5126,10 +5124,10 @@
         <v>149</v>
       </c>
       <c r="B150" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C150" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D150" s="13" t="s">
         <v>19</v>
@@ -5152,10 +5150,10 @@
         <v>150</v>
       </c>
       <c r="B151" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C151" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D151" s="13" t="s">
         <v>19</v>
@@ -5231,12 +5229,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B3" s="17" t="n">
         <f aca="false">COUNTA(Tracker!C2:C151)</f>
@@ -5258,12 +5256,12 @@
       </c>
       <c r="B5" s="17" t="n">
         <f aca="false">COUNTIF(Tracker!I2:I151,"Solved with Help")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B6" s="17" t="n">
         <f aca="false">COUNTIF(Tracker!I2:I151,"Attempted")</f>
@@ -5272,25 +5270,25 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B7" s="17" t="n">
         <f aca="false">COUNTA(Tracker!C2:C151)-COUNTIF(Tracker!I2:I151,"Solved")-COUNTIF(Tracker!I2:I151,"Solved with Help")-COUNTIF(Tracker!I2:I151,"Attempted")</f>
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B8" s="18" t="n">
         <f aca="false">(COUNTIF(Tracker!I2:I151,"Solved")+COUNTIF(Tracker!I2:I151,"Solved with Help"))/COUNTA(Tracker!C2:C151)</f>
-        <v>0.0466666666666667</v>
+        <v>0.0533333333333333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B9" s="17" t="n">
         <f aca="true">COUNTIFS(Tracker!K2:K151,"&lt;="&amp;TODAY(),Tracker!K2:K151,"&lt;&gt;",Tracker!L2:L151,"&lt;&gt;Yes")</f>
@@ -5299,7 +5297,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5331,47 +5329,47 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added design add and search word data structure solution
</commit_message>
<xml_diff>
--- a/neetcode_150_tracker.xlsx
+++ b/neetcode_150_tracker.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Tracker" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="203">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -2836,7 +2836,8 @@
         <v>46221</v>
       </c>
       <c r="K62" s="10" t="n">
-        <v>46247</v>
+        <f aca="false">IF(J62="","",J62+14)</f>
+        <v>46235</v>
       </c>
       <c r="L62" s="11"/>
       <c r="M62" s="8"/>
@@ -2854,13 +2855,24 @@
       <c r="D63" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E63" s="10"/>
-      <c r="F63" s="11"/>
+      <c r="E63" s="10" t="n">
+        <v>46247</v>
+      </c>
+      <c r="F63" s="11" t="s">
+        <v>79</v>
+      </c>
       <c r="G63" s="8"/>
       <c r="H63" s="8"/>
-      <c r="I63" s="11"/>
-      <c r="J63" s="12"/>
-      <c r="K63" s="10"/>
+      <c r="I63" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="J63" s="12" t="n">
+        <v>46247</v>
+      </c>
+      <c r="K63" s="10" t="n">
+        <f aca="false">IF(J63="","",J63+14)</f>
+        <v>46261</v>
+      </c>
       <c r="L63" s="11"/>
       <c r="M63" s="8"/>
     </row>
@@ -2883,7 +2895,10 @@
       <c r="H64" s="8"/>
       <c r="I64" s="11"/>
       <c r="J64" s="12"/>
-      <c r="K64" s="10"/>
+      <c r="K64" s="10" t="str">
+        <f aca="false">IF(J64="","",J64+14)</f>
+        <v/>
+      </c>
       <c r="L64" s="11"/>
       <c r="M64" s="8"/>
     </row>
@@ -5256,7 +5271,7 @@
       </c>
       <c r="B5" s="17" t="n">
         <f aca="false">COUNTIF(Tracker!I2:I151,"Solved with Help")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5274,7 +5289,7 @@
       </c>
       <c r="B7" s="17" t="n">
         <f aca="false">COUNTA(Tracker!C2:C151)-COUNTIF(Tracker!I2:I151,"Solved")-COUNTIF(Tracker!I2:I151,"Solved with Help")-COUNTIF(Tracker!I2:I151,"Attempted")</f>
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5283,7 +5298,7 @@
       </c>
       <c r="B8" s="18" t="n">
         <f aca="false">(COUNTIF(Tracker!I2:I151,"Solved")+COUNTIF(Tracker!I2:I151,"Solved with Help"))/COUNTA(Tracker!C2:C151)</f>
-        <v>0.0533333333333333</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5292,7 +5307,7 @@
       </c>
       <c r="B9" s="17" t="n">
         <f aca="true">COUNTIFS(Tracker!K2:K151,"&lt;="&amp;TODAY(),Tracker!K2:K151,"&lt;&gt;",Tracker!L2:L151,"&lt;&gt;Yes")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
added Word Search II solution
</commit_message>
<xml_diff>
--- a/neetcode_150_tracker.xlsx
+++ b/neetcode_150_tracker.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="203">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -2889,15 +2889,23 @@
       <c r="D64" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="E64" s="10"/>
-      <c r="F64" s="11"/>
+      <c r="E64" s="10" t="n">
+        <v>46249</v>
+      </c>
+      <c r="F64" s="11" t="s">
+        <v>79</v>
+      </c>
       <c r="G64" s="8"/>
       <c r="H64" s="8"/>
-      <c r="I64" s="11"/>
-      <c r="J64" s="12"/>
-      <c r="K64" s="10" t="str">
+      <c r="I64" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="J64" s="12" t="n">
+        <v>46249</v>
+      </c>
+      <c r="K64" s="10" t="n">
         <f aca="false">IF(J64="","",J64+14)</f>
-        <v/>
+        <v>46263</v>
       </c>
       <c r="L64" s="11"/>
       <c r="M64" s="8"/>
@@ -5271,7 +5279,7 @@
       </c>
       <c r="B5" s="17" t="n">
         <f aca="false">COUNTIF(Tracker!I2:I151,"Solved with Help")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5289,7 +5297,7 @@
       </c>
       <c r="B7" s="17" t="n">
         <f aca="false">COUNTA(Tracker!C2:C151)-COUNTIF(Tracker!I2:I151,"Solved")-COUNTIF(Tracker!I2:I151,"Solved with Help")-COUNTIF(Tracker!I2:I151,"Attempted")</f>
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5298,7 +5306,7 @@
       </c>
       <c r="B8" s="18" t="n">
         <f aca="false">(COUNTIF(Tracker!I2:I151,"Solved")+COUNTIF(Tracker!I2:I151,"Solved with Help"))/COUNTA(Tracker!C2:C151)</f>
-        <v>0.06</v>
+        <v>0.0666666666666667</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Added Number Of Islands solution
</commit_message>
<xml_diff>
--- a/neetcode_150_tracker.xlsx
+++ b/neetcode_150_tracker.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="203">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -272,85 +272,85 @@
     <t xml:space="preserve">Binary Tree Maximum Path Sum</t>
   </si>
   <si>
+    <t xml:space="preserve">Serialize and Deserialize Binary Tree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implement Trie (Prefix Tree)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design Add and Search Words Data Structure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Word Search II</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heap / Priority Queue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kth Largest Element in a Stream</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last Stone Weight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K Closest Points to Origin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kth Largest Element in an Array</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Task Scheduler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design Twitter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Find Median from Data Stream</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backtracking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subsets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combination Sum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permutations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subsets II</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combination Sum II</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Word Search</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Palindrome Partitioning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Letter Combinations of a Phone Number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N-Queens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Graphs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of Islands</t>
+  </si>
+  <si>
     <t xml:space="preserve">Solved with Help</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serialize and Deserialize Binary Tree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tries</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implement Trie (Prefix Tree)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design Add and Search Words Data Structure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Word Search II</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heap / Priority Queue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kth Largest Element in a Stream</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last Stone Weight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K Closest Points to Origin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kth Largest Element in an Array</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Task Scheduler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design Twitter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Find Median from Data Stream</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Backtracking</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subsets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Combination Sum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permutations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subsets II</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Combination Sum II</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Word Search</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Palindrome Partitioning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Letter Combinations of a Phone Number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N-Queens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Graphs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of Islands</t>
   </si>
   <si>
     <t xml:space="preserve">Clone Graph</t>
@@ -2764,14 +2764,12 @@
       <c r="G60" s="8"/>
       <c r="H60" s="8"/>
       <c r="I60" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="J60" s="12" t="n">
-        <v>46217</v>
-      </c>
-      <c r="K60" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="J60" s="12"/>
+      <c r="K60" s="10" t="str">
         <f aca="false">IF(J60="","",J60+14)</f>
-        <v>46231</v>
+        <v/>
       </c>
       <c r="L60" s="11"/>
       <c r="M60" s="8"/>
@@ -2784,7 +2782,7 @@
         <v>66</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D61" s="14" t="s">
         <v>31</v>
@@ -2793,7 +2791,7 @@
         <v>46218</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G61" s="8"/>
       <c r="H61" s="8"/>
@@ -2813,10 +2811,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C62" s="8" t="s">
         <v>86</v>
-      </c>
-      <c r="C62" s="8" t="s">
-        <v>87</v>
       </c>
       <c r="D62" s="13" t="s">
         <v>19</v>
@@ -2830,14 +2828,12 @@
       <c r="G62" s="8"/>
       <c r="H62" s="8"/>
       <c r="I62" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="J62" s="12" t="n">
-        <v>46221</v>
-      </c>
-      <c r="K62" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="J62" s="12"/>
+      <c r="K62" s="10" t="str">
         <f aca="false">IF(J62="","",J62+14)</f>
-        <v>46235</v>
+        <v/>
       </c>
       <c r="L62" s="11"/>
       <c r="M62" s="8"/>
@@ -2847,10 +2843,10 @@
         <v>62</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D63" s="13" t="s">
         <v>19</v>
@@ -2864,14 +2860,12 @@
       <c r="G63" s="8"/>
       <c r="H63" s="8"/>
       <c r="I63" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="J63" s="12" t="n">
-        <v>46247</v>
-      </c>
-      <c r="K63" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="J63" s="12"/>
+      <c r="K63" s="10" t="str">
         <f aca="false">IF(J63="","",J63+14)</f>
-        <v>46261</v>
+        <v/>
       </c>
       <c r="L63" s="11"/>
       <c r="M63" s="8"/>
@@ -2881,10 +2875,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D64" s="14" t="s">
         <v>31</v>
@@ -2898,14 +2892,12 @@
       <c r="G64" s="8"/>
       <c r="H64" s="8"/>
       <c r="I64" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="J64" s="12" t="n">
-        <v>46249</v>
-      </c>
-      <c r="K64" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="J64" s="12"/>
+      <c r="K64" s="10" t="str">
         <f aca="false">IF(J64="","",J64+14)</f>
-        <v>46263</v>
+        <v/>
       </c>
       <c r="L64" s="11"/>
       <c r="M64" s="8"/>
@@ -2915,10 +2907,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="C65" s="8" t="s">
         <v>90</v>
-      </c>
-      <c r="C65" s="8" t="s">
-        <v>91</v>
       </c>
       <c r="D65" s="9" t="s">
         <v>15</v>
@@ -2941,10 +2933,10 @@
         <v>65</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D66" s="9" t="s">
         <v>15</v>
@@ -2967,10 +2959,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D67" s="13" t="s">
         <v>19</v>
@@ -2993,10 +2985,10 @@
         <v>67</v>
       </c>
       <c r="B68" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C68" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D68" s="13" t="s">
         <v>19</v>
@@ -3019,10 +3011,10 @@
         <v>68</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D69" s="13" t="s">
         <v>19</v>
@@ -3045,10 +3037,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C70" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D70" s="13" t="s">
         <v>19</v>
@@ -3071,10 +3063,10 @@
         <v>70</v>
       </c>
       <c r="B71" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D71" s="14" t="s">
         <v>31</v>
@@ -3103,10 +3095,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="C72" s="8" t="s">
         <v>98</v>
-      </c>
-      <c r="C72" s="8" t="s">
-        <v>99</v>
       </c>
       <c r="D72" s="13" t="s">
         <v>19</v>
@@ -3129,10 +3121,10 @@
         <v>72</v>
       </c>
       <c r="B73" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C73" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D73" s="13" t="s">
         <v>19</v>
@@ -3148,12 +3140,10 @@
       <c r="I73" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="J73" s="12" t="n">
-        <v>46221</v>
-      </c>
-      <c r="K73" s="10" t="n">
+      <c r="J73" s="12"/>
+      <c r="K73" s="10" t="str">
         <f aca="false">IF(J73="","",J73+14)</f>
-        <v>46235</v>
+        <v/>
       </c>
       <c r="L73" s="11"/>
       <c r="M73" s="8"/>
@@ -3163,10 +3153,10 @@
         <v>73</v>
       </c>
       <c r="B74" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C74" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D74" s="13" t="s">
         <v>19</v>
@@ -3189,10 +3179,10 @@
         <v>74</v>
       </c>
       <c r="B75" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D75" s="13" t="s">
         <v>19</v>
@@ -3215,10 +3205,10 @@
         <v>75</v>
       </c>
       <c r="B76" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D76" s="13" t="s">
         <v>19</v>
@@ -3241,10 +3231,10 @@
         <v>76</v>
       </c>
       <c r="B77" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D77" s="13" t="s">
         <v>19</v>
@@ -3258,14 +3248,12 @@
       <c r="G77" s="8"/>
       <c r="H77" s="8"/>
       <c r="I77" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="J77" s="12" t="n">
-        <v>46231</v>
-      </c>
-      <c r="K77" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="J77" s="12"/>
+      <c r="K77" s="10" t="str">
         <f aca="false">IF(J77="","",J77+14)</f>
-        <v>46245</v>
+        <v/>
       </c>
       <c r="L77" s="11"/>
       <c r="M77" s="8"/>
@@ -3275,10 +3263,10 @@
         <v>77</v>
       </c>
       <c r="B78" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D78" s="13" t="s">
         <v>19</v>
@@ -3301,10 +3289,10 @@
         <v>78</v>
       </c>
       <c r="B79" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D79" s="13" t="s">
         <v>19</v>
@@ -3327,10 +3315,10 @@
         <v>79</v>
       </c>
       <c r="B80" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C80" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D80" s="14" t="s">
         <v>31</v>
@@ -3353,23 +3341,31 @@
         <v>80</v>
       </c>
       <c r="B81" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C81" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="C81" s="8" t="s">
-        <v>109</v>
-      </c>
       <c r="D81" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E81" s="10"/>
-      <c r="F81" s="11"/>
+      <c r="E81" s="10" t="n">
+        <v>46257</v>
+      </c>
+      <c r="F81" s="11" t="s">
+        <v>79</v>
+      </c>
       <c r="G81" s="8"/>
       <c r="H81" s="8"/>
-      <c r="I81" s="11"/>
-      <c r="J81" s="12"/>
-      <c r="K81" s="10" t="str">
+      <c r="I81" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="J81" s="12" t="n">
+        <v>46257</v>
+      </c>
+      <c r="K81" s="10" t="n">
         <f aca="false">IF(J81="","",J81+14)</f>
-        <v/>
+        <v>46271</v>
       </c>
       <c r="L81" s="11"/>
       <c r="M81" s="8"/>
@@ -3379,7 +3375,7 @@
         <v>81</v>
       </c>
       <c r="B82" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C82" s="8" t="s">
         <v>110</v>
@@ -3405,7 +3401,7 @@
         <v>82</v>
       </c>
       <c r="B83" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C83" s="8" t="s">
         <v>111</v>
@@ -3431,7 +3427,7 @@
         <v>83</v>
       </c>
       <c r="B84" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C84" s="8" t="s">
         <v>112</v>
@@ -3457,7 +3453,7 @@
         <v>84</v>
       </c>
       <c r="B85" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C85" s="8" t="s">
         <v>113</v>
@@ -3483,7 +3479,7 @@
         <v>85</v>
       </c>
       <c r="B86" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C86" s="8" t="s">
         <v>114</v>
@@ -3509,7 +3505,7 @@
         <v>86</v>
       </c>
       <c r="B87" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C87" s="8" t="s">
         <v>115</v>
@@ -3535,7 +3531,7 @@
         <v>87</v>
       </c>
       <c r="B88" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C88" s="8" t="s">
         <v>116</v>
@@ -3561,7 +3557,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C89" s="8" t="s">
         <v>117</v>
@@ -3587,7 +3583,7 @@
         <v>89</v>
       </c>
       <c r="B90" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C90" s="8" t="s">
         <v>118</v>
@@ -3613,7 +3609,7 @@
         <v>90</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C91" s="8" t="s">
         <v>119</v>
@@ -3639,7 +3635,7 @@
         <v>91</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C92" s="8" t="s">
         <v>120</v>
@@ -3665,7 +3661,7 @@
         <v>92</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C93" s="8" t="s">
         <v>121</v>
@@ -5270,16 +5266,16 @@
       </c>
       <c r="B4" s="17" t="n">
         <f aca="false">COUNTIF(Tracker!I2:I151,"Solved")</f>
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>83</v>
+        <v>109</v>
       </c>
       <c r="B5" s="17" t="n">
         <f aca="false">COUNTIF(Tracker!I2:I151,"Solved with Help")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5297,7 +5293,7 @@
       </c>
       <c r="B7" s="17" t="n">
         <f aca="false">COUNTA(Tracker!C2:C151)-COUNTIF(Tracker!I2:I151,"Solved")-COUNTIF(Tracker!I2:I151,"Solved with Help")-COUNTIF(Tracker!I2:I151,"Attempted")</f>
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5306,7 +5302,7 @@
       </c>
       <c r="B8" s="18" t="n">
         <f aca="false">(COUNTIF(Tracker!I2:I151,"Solved")+COUNTIF(Tracker!I2:I151,"Solved with Help"))/COUNTA(Tracker!C2:C151)</f>
-        <v>0.0666666666666667</v>
+        <v>0.0733333333333333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5315,7 +5311,7 @@
       </c>
       <c r="B9" s="17" t="n">
         <f aca="true">COUNTIFS(Tracker!K2:K151,"&lt;="&amp;TODAY(),Tracker!K2:K151,"&lt;&gt;",Tracker!L2:L151,"&lt;&gt;Yes")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5338,7 +5334,7 @@
       </c>
       <c r="B13" s="17" t="str">
         <f aca="false">COUNTIFS(Tracker!D2:D151,"Medium",Tracker!I2:I151,"Solved")&amp;"/"&amp;COUNTIF(Tracker!D2:D151,"Medium")</f>
-        <v>3/101</v>
+        <v>6/101</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5347,7 +5343,7 @@
       </c>
       <c r="B14" s="17" t="str">
         <f aca="false">COUNTIFS(Tracker!D2:D151,"Hard",Tracker!I2:I151,"Solved")&amp;"/"&amp;COUNTIF(Tracker!D2:D151,"Hard")</f>
-        <v>2/21</v>
+        <v>4/21</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>